<commit_message>
argus do sul -> meripurpuratus
</commit_message>
<xml_diff>
--- a/dados/Ocorrências Literatura.xlsx
+++ b/dados/Ocorrências Literatura.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Cofres Obsidian\Mar Aberto\Laboratório\lagostas_carapaca\Modelagem\Dados produzidos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Cofres Obsidian\Mar Aberto\Laboratório\analysis-panulirus\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{252403E3-8A1B-4779-9C8E-8421F69929CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20768F61-CD33-49AC-88B1-63C9585045F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5205" yWindow="4215" windowWidth="16140" windowHeight="7515" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ocorrências Panulirus" sheetId="1" r:id="rId1"/>
@@ -3399,6 +3399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:R481"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3480,7 +3481,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>18</v>
@@ -3544,7 +3545,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>26</v>
@@ -3608,7 +3609,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>26</v>
@@ -3672,7 +3673,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>26</v>
@@ -3736,7 +3737,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>26</v>
@@ -3800,7 +3801,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>26</v>
@@ -3859,7 +3860,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -3923,7 +3924,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -3987,7 +3988,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -4051,7 +4052,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -4115,7 +4116,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -4179,7 +4180,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="16.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -4243,7 +4244,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -4307,7 +4308,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -4371,7 +4372,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -4435,7 +4436,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -4499,7 +4500,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -4563,7 +4564,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -4627,7 +4628,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -4691,7 +4692,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -4755,7 +4756,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -4819,7 +4820,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -4883,7 +4884,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -4947,7 +4948,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -5011,7 +5012,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -5075,7 +5076,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -5139,7 +5140,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -5203,7 +5204,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -5267,7 +5268,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -5336,7 +5337,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>18</v>
@@ -5400,7 +5401,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>18</v>
@@ -5464,7 +5465,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>18</v>
@@ -5523,7 +5524,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -5587,7 +5588,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -5651,7 +5652,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -5715,7 +5716,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -5779,7 +5780,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -5843,7 +5844,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -5907,7 +5908,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -5976,7 +5977,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>26</v>
@@ -6035,7 +6036,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -6099,7 +6100,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="43" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -6168,7 +6169,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>26</v>
@@ -6227,7 +6228,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="45" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -6291,7 +6292,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="46" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -6355,7 +6356,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -6419,7 +6420,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -6483,7 +6484,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -6547,7 +6548,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -6616,7 +6617,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>26</v>
@@ -6680,7 +6681,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>26</v>
@@ -6739,7 +6740,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -6803,7 +6804,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -6867,7 +6868,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="55" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -6931,7 +6932,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -7000,7 +7001,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>26</v>
@@ -7064,7 +7065,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>26</v>
@@ -7128,7 +7129,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>26</v>
@@ -7187,7 +7188,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -7251,7 +7252,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="61" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -7315,7 +7316,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="62" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -7379,7 +7380,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="63" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -7443,7 +7444,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="64" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -7507,7 +7508,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="65" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -7576,7 +7577,7 @@
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>26</v>
@@ -7635,7 +7636,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="67" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -7699,7 +7700,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -7763,7 +7764,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="69" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>68</v>
       </c>
@@ -7827,7 +7828,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>69</v>
       </c>
@@ -7891,7 +7892,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="71" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -7955,7 +7956,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="72" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -8024,7 +8025,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>18</v>
@@ -8083,7 +8084,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -8147,7 +8148,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -8211,7 +8212,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="76" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>75</v>
       </c>
@@ -8275,7 +8276,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="77" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>76</v>
       </c>
@@ -8344,7 +8345,7 @@
         <v>77</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>26</v>
@@ -8408,7 +8409,7 @@
         <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>26</v>
@@ -8472,7 +8473,7 @@
         <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>26</v>
@@ -8664,7 +8665,7 @@
         <v>82</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>26</v>
@@ -9176,7 +9177,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>18</v>
@@ -9240,7 +9241,7 @@
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>26</v>
@@ -9299,7 +9300,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="93" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>92</v>
       </c>
@@ -9363,7 +9364,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="94" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>93</v>
       </c>
@@ -9496,7 +9497,7 @@
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>26</v>
@@ -9560,7 +9561,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>26</v>
@@ -9624,7 +9625,7 @@
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C98" s="1" t="s">
         <v>18</v>
@@ -9688,7 +9689,7 @@
         <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>18</v>
@@ -9752,7 +9753,7 @@
         <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>26</v>
@@ -9816,7 +9817,7 @@
         <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>18</v>
@@ -9880,7 +9881,7 @@
         <v>101</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>26</v>
@@ -9944,7 +9945,7 @@
         <v>102</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>26</v>
@@ -10008,7 +10009,7 @@
         <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>26</v>
@@ -10072,7 +10073,7 @@
         <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>26</v>
@@ -10136,7 +10137,7 @@
         <v>105</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>26</v>
@@ -10200,7 +10201,7 @@
         <v>106</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>26</v>
@@ -10264,7 +10265,7 @@
         <v>107</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>26</v>
@@ -10328,7 +10329,7 @@
         <v>108</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>26</v>
@@ -10835,7 +10836,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="117" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
         <v>116</v>
       </c>
@@ -10899,7 +10900,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="118" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
         <v>117</v>
       </c>
@@ -10963,7 +10964,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="119" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
         <v>118</v>
       </c>
@@ -11027,7 +11028,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="120" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
         <v>119</v>
       </c>
@@ -11091,7 +11092,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="121" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
         <v>120</v>
       </c>
@@ -11155,7 +11156,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="122" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
         <v>121</v>
       </c>
@@ -11219,7 +11220,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="123" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="1">
         <v>122</v>
       </c>
@@ -11283,7 +11284,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="124" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1">
         <v>123</v>
       </c>
@@ -11352,7 +11353,7 @@
         <v>124</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>26</v>
@@ -11416,7 +11417,7 @@
         <v>125</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>26</v>
@@ -11480,7 +11481,7 @@
         <v>126</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>26</v>
@@ -11544,7 +11545,7 @@
         <v>127</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>26</v>
@@ -11608,7 +11609,7 @@
         <v>128</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>26</v>
@@ -11672,7 +11673,7 @@
         <v>129</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>26</v>
@@ -11736,7 +11737,7 @@
         <v>130</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>26</v>
@@ -11800,7 +11801,7 @@
         <v>131</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>26</v>
@@ -11859,7 +11860,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="133" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="1">
         <v>132</v>
       </c>
@@ -11923,7 +11924,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="134" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="1">
         <v>133</v>
       </c>
@@ -11987,7 +11988,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="135" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="1">
         <v>134</v>
       </c>
@@ -12051,7 +12052,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="136" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="1">
         <v>135</v>
       </c>
@@ -12115,7 +12116,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="137" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="1">
         <v>136</v>
       </c>
@@ -12179,7 +12180,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="138" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="1">
         <v>137</v>
       </c>
@@ -12243,7 +12244,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="139" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="1">
         <v>138</v>
       </c>
@@ -12312,7 +12313,7 @@
         <v>139</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>26</v>
@@ -12376,7 +12377,7 @@
         <v>140</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C141" s="1" t="s">
         <v>26</v>
@@ -12435,7 +12436,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="142" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="1">
         <v>141</v>
       </c>
@@ -12499,7 +12500,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="143" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="1">
         <v>142</v>
       </c>
@@ -12563,7 +12564,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="144" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="1">
         <v>143</v>
       </c>
@@ -12627,7 +12628,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="145" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="1">
         <v>144</v>
       </c>
@@ -12691,7 +12692,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="146" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="1">
         <v>145</v>
       </c>
@@ -12755,7 +12756,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="147" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="1">
         <v>146</v>
       </c>
@@ -12819,7 +12820,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="148" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="1">
         <v>147</v>
       </c>
@@ -12883,7 +12884,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="149" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="1">
         <v>148</v>
       </c>
@@ -12947,7 +12948,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="150" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="1">
         <v>149</v>
       </c>
@@ -13011,7 +13012,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="151" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="1">
         <v>150</v>
       </c>
@@ -13075,7 +13076,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="152" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="1">
         <v>151</v>
       </c>
@@ -13139,7 +13140,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="153" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="1">
         <v>152</v>
       </c>
@@ -13203,7 +13204,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="154" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="1">
         <v>153</v>
       </c>
@@ -13267,7 +13268,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="155" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="1">
         <v>154</v>
       </c>
@@ -13331,7 +13332,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="156" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="1">
         <v>155</v>
       </c>
@@ -13395,7 +13396,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="157" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="1">
         <v>156</v>
       </c>
@@ -13459,7 +13460,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="158" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="1">
         <v>157</v>
       </c>
@@ -13523,7 +13524,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="159" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="1">
         <v>158</v>
       </c>
@@ -13587,7 +13588,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="160" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="1">
         <v>159</v>
       </c>
@@ -13651,7 +13652,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="161" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="1">
         <v>160</v>
       </c>
@@ -13715,7 +13716,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="162" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" s="1">
         <v>161</v>
       </c>
@@ -13779,7 +13780,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="163" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="1">
         <v>162</v>
       </c>
@@ -13843,7 +13844,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="164" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="1">
         <v>163</v>
       </c>
@@ -13907,7 +13908,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="165" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" s="1">
         <v>164</v>
       </c>
@@ -13971,7 +13972,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="166" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="1">
         <v>165</v>
       </c>
@@ -14035,7 +14036,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="167" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="1">
         <v>166</v>
       </c>
@@ -14104,7 +14105,7 @@
         <v>167</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>26</v>
@@ -14168,7 +14169,7 @@
         <v>168</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C169" s="1" t="s">
         <v>26</v>
@@ -14232,7 +14233,7 @@
         <v>169</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C170" s="1" t="s">
         <v>26</v>
@@ -14296,7 +14297,7 @@
         <v>170</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C171" s="1" t="s">
         <v>26</v>
@@ -14360,7 +14361,7 @@
         <v>171</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>26</v>
@@ -14424,7 +14425,7 @@
         <v>172</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C173" s="1" t="s">
         <v>26</v>
@@ -14488,7 +14489,7 @@
         <v>173</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C174" s="1" t="s">
         <v>26</v>
@@ -14552,7 +14553,7 @@
         <v>174</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C175" s="1" t="s">
         <v>26</v>
@@ -14616,7 +14617,7 @@
         <v>175</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C176" s="1" t="s">
         <v>26</v>
@@ -14680,7 +14681,7 @@
         <v>176</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C177" s="1" t="s">
         <v>26</v>
@@ -14744,7 +14745,7 @@
         <v>177</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C178" s="1" t="s">
         <v>26</v>
@@ -14808,7 +14809,7 @@
         <v>178</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C179" s="1" t="s">
         <v>26</v>
@@ -18003,7 +18004,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="229" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" s="1">
         <v>228</v>
       </c>
@@ -18067,7 +18068,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="230" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" s="1">
         <v>229</v>
       </c>
@@ -18131,7 +18132,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="231" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" s="1">
         <v>230</v>
       </c>
@@ -18195,7 +18196,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="232" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" s="1">
         <v>231</v>
       </c>
@@ -18259,7 +18260,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="233" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" s="1">
         <v>232</v>
       </c>
@@ -18323,7 +18324,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="234" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" s="1">
         <v>233</v>
       </c>
@@ -19923,7 +19924,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="259" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:18" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A259" s="1">
         <v>258</v>
       </c>
@@ -19987,7 +19988,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="260" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:18" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A260" s="1">
         <v>259</v>
       </c>
@@ -20051,7 +20052,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="261" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A261" s="1">
         <v>260</v>
       </c>
@@ -20115,7 +20116,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="262" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:18" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A262" s="1">
         <v>261</v>
       </c>
@@ -20179,7 +20180,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="263" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:18" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A263" s="1">
         <v>262</v>
       </c>
@@ -20243,7 +20244,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="264" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:18" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A264" s="1">
         <v>263</v>
       </c>
@@ -20307,7 +20308,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="265" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:18" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A265" s="1">
         <v>264</v>
       </c>
@@ -20371,7 +20372,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="266" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:18" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A266" s="1">
         <v>265</v>
       </c>
@@ -20435,7 +20436,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="267" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:18" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A267" s="1">
         <v>266</v>
       </c>
@@ -20499,7 +20500,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="268" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:18" ht="16.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A268" s="1">
         <v>267</v>
       </c>
@@ -20563,7 +20564,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="269" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:18" ht="16.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A269" s="1">
         <v>268</v>
       </c>
@@ -20627,7 +20628,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="270" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:18" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A270" s="1">
         <v>269</v>
       </c>
@@ -20691,7 +20692,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="271" spans="1:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:18" ht="16.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A271" s="1">
         <v>270</v>
       </c>
@@ -20755,7 +20756,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="272" spans="1:18" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:18" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A272" s="1">
         <v>271</v>
       </c>
@@ -24083,7 +24084,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="324" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A324" s="1">
         <v>323</v>
       </c>
@@ -24147,7 +24148,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="325" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A325" s="1">
         <v>324</v>
       </c>
@@ -24211,7 +24212,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="326" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A326" s="1">
         <v>325</v>
       </c>
@@ -24275,7 +24276,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="327" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A327" s="1">
         <v>326</v>
       </c>
@@ -24339,7 +24340,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="328" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A328" s="1">
         <v>327</v>
       </c>
@@ -24403,7 +24404,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="329" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A329" s="1">
         <v>328</v>
       </c>
@@ -24467,7 +24468,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="330" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A330" s="1">
         <v>329</v>
       </c>
@@ -24531,7 +24532,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="331" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A331" s="1">
         <v>330</v>
       </c>
@@ -24595,7 +24596,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="332" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A332" s="1">
         <v>331</v>
       </c>
@@ -24659,7 +24660,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="333" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A333" s="1">
         <v>332</v>
       </c>
@@ -24723,7 +24724,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="334" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A334" s="1">
         <v>333</v>
       </c>
@@ -24787,7 +24788,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="335" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A335" s="1">
         <v>334</v>
       </c>
@@ -24851,7 +24852,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="336" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A336" s="1">
         <v>335</v>
       </c>
@@ -24915,7 +24916,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="337" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A337" s="1">
         <v>336</v>
       </c>
@@ -24979,7 +24980,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="338" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A338" s="1">
         <v>337</v>
       </c>
@@ -25043,7 +25044,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="339" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A339" s="1">
         <v>338</v>
       </c>
@@ -25107,7 +25108,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="340" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A340" s="1">
         <v>339</v>
       </c>
@@ -25171,7 +25172,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="341" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A341" s="1">
         <v>340</v>
       </c>
@@ -25235,7 +25236,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="342" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A342" s="1">
         <v>341</v>
       </c>
@@ -25299,7 +25300,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="343" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A343" s="1">
         <v>342</v>
       </c>
@@ -25363,7 +25364,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="344" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A344" s="1">
         <v>343</v>
       </c>
@@ -25427,7 +25428,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="345" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A345" s="1">
         <v>344</v>
       </c>
@@ -25491,7 +25492,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="346" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A346" s="1">
         <v>345</v>
       </c>
@@ -25555,7 +25556,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="347" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A347" s="1">
         <v>346</v>
       </c>
@@ -25619,7 +25620,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="348" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A348" s="1">
         <v>347</v>
       </c>
@@ -25683,7 +25684,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="349" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A349" s="1">
         <v>348</v>
       </c>
@@ -25747,7 +25748,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="350" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A350" s="1">
         <v>349</v>
       </c>
@@ -25811,7 +25812,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="351" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A351" s="1">
         <v>350</v>
       </c>
@@ -25875,7 +25876,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="352" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A352" s="1">
         <v>351</v>
       </c>
@@ -25939,7 +25940,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="353" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A353" s="1">
         <v>352</v>
       </c>
@@ -26003,7 +26004,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="354" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A354" s="1">
         <v>353</v>
       </c>
@@ -26067,7 +26068,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="355" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A355" s="1">
         <v>354</v>
       </c>
@@ -26131,7 +26132,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="356" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A356" s="1">
         <v>355</v>
       </c>
@@ -26195,7 +26196,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="357" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A357" s="1">
         <v>356</v>
       </c>
@@ -26259,7 +26260,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="358" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A358" s="1">
         <v>357</v>
       </c>
@@ -26323,7 +26324,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="359" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A359" s="1">
         <v>358</v>
       </c>
@@ -26387,7 +26388,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="360" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A360" s="1">
         <v>359</v>
       </c>
@@ -26451,7 +26452,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="361" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A361" s="1">
         <v>360</v>
       </c>
@@ -26515,7 +26516,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="362" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A362" s="1">
         <v>361</v>
       </c>
@@ -26579,7 +26580,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="363" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A363" s="1">
         <v>362</v>
       </c>
@@ -26643,7 +26644,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="364" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A364" s="1">
         <v>363</v>
       </c>
@@ -26707,7 +26708,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="365" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A365" s="1">
         <v>364</v>
       </c>
@@ -26771,7 +26772,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="366" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A366" s="1">
         <v>365</v>
       </c>
@@ -26835,7 +26836,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="367" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A367" s="1">
         <v>366</v>
       </c>
@@ -26899,7 +26900,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="368" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A368" s="1">
         <v>367</v>
       </c>
@@ -26963,7 +26964,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="369" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A369" s="1">
         <v>368</v>
       </c>
@@ -27027,7 +27028,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="370" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A370" s="1">
         <v>369</v>
       </c>
@@ -27091,7 +27092,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="371" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A371" s="1">
         <v>370</v>
       </c>
@@ -27155,7 +27156,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="372" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A372" s="1">
         <v>371</v>
       </c>
@@ -27219,7 +27220,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="373" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A373" s="1">
         <v>372</v>
       </c>
@@ -27283,7 +27284,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="374" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A374" s="1">
         <v>373</v>
       </c>
@@ -27347,7 +27348,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="375" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A375" s="1">
         <v>374</v>
       </c>
@@ -27411,7 +27412,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="376" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A376" s="1">
         <v>375</v>
       </c>
@@ -27475,7 +27476,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="377" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A377" s="1">
         <v>376</v>
       </c>
@@ -27539,7 +27540,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="378" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A378" s="1">
         <v>377</v>
       </c>
@@ -27603,7 +27604,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="379" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A379" s="1">
         <v>378</v>
       </c>
@@ -27667,7 +27668,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="380" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A380" s="1">
         <v>379</v>
       </c>
@@ -27731,7 +27732,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="381" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A381" s="1">
         <v>380</v>
       </c>
@@ -27795,7 +27796,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="382" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A382" s="1">
         <v>381</v>
       </c>
@@ -27859,7 +27860,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="383" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A383" s="1">
         <v>382</v>
       </c>
@@ -27923,7 +27924,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="384" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A384" s="1">
         <v>383</v>
       </c>
@@ -27987,7 +27988,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="385" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A385" s="1">
         <v>384</v>
       </c>
@@ -28051,7 +28052,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="386" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A386" s="1">
         <v>385</v>
       </c>
@@ -28115,7 +28116,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="387" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A387" s="1">
         <v>386</v>
       </c>
@@ -28179,7 +28180,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="388" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A388" s="1">
         <v>387</v>
       </c>
@@ -28243,7 +28244,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="389" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A389" s="1">
         <v>388</v>
       </c>
@@ -28307,7 +28308,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="390" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A390" s="1">
         <v>389</v>
       </c>
@@ -28371,7 +28372,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="391" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A391" s="1">
         <v>390</v>
       </c>
@@ -28435,7 +28436,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="392" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A392" s="1">
         <v>391</v>
       </c>
@@ -28499,7 +28500,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="393" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A393" s="1">
         <v>392</v>
       </c>
@@ -28563,7 +28564,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="394" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A394" s="1">
         <v>393</v>
       </c>
@@ -28627,7 +28628,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="395" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A395" s="1">
         <v>394</v>
       </c>
@@ -28691,7 +28692,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="396" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A396" s="1">
         <v>395</v>
       </c>
@@ -28755,7 +28756,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="397" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A397" s="1">
         <v>396</v>
       </c>
@@ -28819,7 +28820,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="398" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A398" s="1">
         <v>397</v>
       </c>
@@ -28883,7 +28884,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="399" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A399" s="1">
         <v>398</v>
       </c>
@@ -28947,7 +28948,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="400" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A400" s="1">
         <v>399</v>
       </c>
@@ -29011,7 +29012,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="401" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A401" s="1">
         <v>400</v>
       </c>
@@ -29075,7 +29076,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="402" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A402" s="1">
         <v>401</v>
       </c>
@@ -29139,7 +29140,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="403" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A403" s="1">
         <v>402</v>
       </c>
@@ -29203,7 +29204,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="404" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A404" s="1">
         <v>403</v>
       </c>
@@ -29267,7 +29268,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="405" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A405" s="1">
         <v>404</v>
       </c>
@@ -29331,7 +29332,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="406" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A406" s="1">
         <v>405</v>
       </c>
@@ -29395,7 +29396,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="407" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A407" s="1">
         <v>406</v>
       </c>
@@ -29459,7 +29460,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="408" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A408" s="1">
         <v>407</v>
       </c>
@@ -29523,7 +29524,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="409" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A409" s="1">
         <v>408</v>
       </c>
@@ -29587,7 +29588,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="410" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A410" s="1">
         <v>409</v>
       </c>
@@ -29651,7 +29652,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="411" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A411" s="1">
         <v>410</v>
       </c>
@@ -29715,7 +29716,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="412" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A412" s="1">
         <v>411</v>
       </c>
@@ -29779,7 +29780,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="413" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A413" s="1">
         <v>412</v>
       </c>
@@ -29843,7 +29844,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="414" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A414" s="1">
         <v>413</v>
       </c>
@@ -29907,7 +29908,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="415" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A415" s="1">
         <v>414</v>
       </c>
@@ -29971,7 +29972,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="416" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A416" s="1">
         <v>415</v>
       </c>
@@ -30035,7 +30036,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="417" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A417" s="1">
         <v>416</v>
       </c>
@@ -30099,7 +30100,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="418" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A418" s="1">
         <v>417</v>
       </c>
@@ -30163,7 +30164,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="419" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A419" s="1">
         <v>418</v>
       </c>
@@ -30227,7 +30228,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="420" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A420" s="1">
         <v>419</v>
       </c>
@@ -30291,7 +30292,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="421" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A421" s="1">
         <v>420</v>
       </c>
@@ -30355,7 +30356,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="422" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A422" s="1">
         <v>421</v>
       </c>
@@ -30419,7 +30420,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="423" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A423" s="1">
         <v>422</v>
       </c>
@@ -30483,7 +30484,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="424" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A424" s="1">
         <v>423</v>
       </c>
@@ -30547,7 +30548,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="425" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A425" s="1">
         <v>424</v>
       </c>
@@ -30611,7 +30612,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="426" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A426" s="1">
         <v>425</v>
       </c>
@@ -30675,7 +30676,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="427" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A427" s="1">
         <v>426</v>
       </c>
@@ -30739,7 +30740,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="428" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A428" s="1">
         <v>427</v>
       </c>
@@ -30803,7 +30804,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="429" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A429" s="1">
         <v>428</v>
       </c>
@@ -30867,7 +30868,7 @@
         <v>771</v>
       </c>
     </row>
-    <row r="430" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A430" s="1">
         <v>429</v>
       </c>
@@ -30931,7 +30932,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="431" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A431" s="1">
         <v>430</v>
       </c>
@@ -30995,7 +30996,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="432" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A432" s="1">
         <v>431</v>
       </c>
@@ -31059,7 +31060,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="433" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A433" s="1">
         <v>432</v>
       </c>
@@ -31123,7 +31124,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="434" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A434" s="1">
         <v>433</v>
       </c>
@@ -31187,7 +31188,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="435" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A435" s="1">
         <v>434</v>
       </c>
@@ -31251,7 +31252,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="436" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A436" s="1">
         <v>435</v>
       </c>
@@ -31315,7 +31316,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="437" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A437" s="1">
         <v>436</v>
       </c>
@@ -31379,7 +31380,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="438" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A438" s="1">
         <v>437</v>
       </c>
@@ -31443,7 +31444,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="439" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A439" s="1">
         <v>438</v>
       </c>
@@ -31507,7 +31508,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="440" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A440" s="1">
         <v>439</v>
       </c>
@@ -31571,7 +31572,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="441" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A441" s="1">
         <v>440</v>
       </c>
@@ -31635,7 +31636,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="442" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A442" s="1">
         <v>441</v>
       </c>
@@ -31699,7 +31700,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="443" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A443" s="1">
         <v>442</v>
       </c>
@@ -31763,7 +31764,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="444" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A444" s="1">
         <v>443</v>
       </c>
@@ -31827,7 +31828,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="445" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A445" s="1">
         <v>444</v>
       </c>
@@ -31891,7 +31892,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="446" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A446" s="1">
         <v>445</v>
       </c>
@@ -31955,7 +31956,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="447" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A447" s="1">
         <v>446</v>
       </c>
@@ -32019,7 +32020,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="448" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A448" s="1">
         <v>447</v>
       </c>
@@ -32083,7 +32084,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="449" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A449" s="1">
         <v>448</v>
       </c>
@@ -32147,7 +32148,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="450" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A450" s="1">
         <v>449</v>
       </c>
@@ -32211,7 +32212,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="451" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A451" s="1">
         <v>450</v>
       </c>
@@ -32275,7 +32276,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="452" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A452" s="1">
         <v>451</v>
       </c>
@@ -32339,7 +32340,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="453" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A453" s="1">
         <v>452</v>
       </c>
@@ -32403,7 +32404,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="454" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A454" s="1">
         <v>453</v>
       </c>
@@ -32467,7 +32468,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="455" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A455" s="1">
         <v>454</v>
       </c>
@@ -32531,7 +32532,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="456" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A456" s="1">
         <v>455</v>
       </c>
@@ -32595,7 +32596,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="457" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A457" s="1">
         <v>456</v>
       </c>
@@ -32659,7 +32660,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="458" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A458" s="1">
         <v>457</v>
       </c>
@@ -32723,7 +32724,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="459" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A459" s="1">
         <v>458</v>
       </c>
@@ -32787,7 +32788,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="460" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A460" s="1">
         <v>459</v>
       </c>
@@ -32851,7 +32852,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="461" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A461" s="1">
         <v>460</v>
       </c>
@@ -32915,7 +32916,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="462" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A462" s="1">
         <v>461</v>
       </c>
@@ -32979,7 +32980,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="463" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A463" s="1">
         <v>462</v>
       </c>
@@ -33043,7 +33044,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="464" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:18" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A464" s="1">
         <v>463</v>
       </c>
@@ -33107,7 +33108,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="465" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="465" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="G465"/>
       <c r="J465" s="1" t="e">
         <f t="shared" si="123"/>
@@ -33142,7 +33143,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="466" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="466" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="G466"/>
       <c r="J466" s="1" t="e">
         <f t="shared" si="123"/>
@@ -33177,7 +33178,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="467" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="467" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="G467"/>
       <c r="J467" s="1" t="e">
         <f t="shared" si="123"/>
@@ -33212,7 +33213,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="468" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="468" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="G468"/>
       <c r="J468" s="1" t="e">
         <f t="shared" si="123"/>
@@ -33247,7 +33248,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="469" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="469" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="G469"/>
       <c r="J469" s="1" t="e">
         <f t="shared" si="123"/>
@@ -33282,7 +33283,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="470" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="470" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="G470"/>
       <c r="J470" s="1" t="e">
         <f t="shared" si="123"/>
@@ -33317,7 +33318,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="471" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="471" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="G471"/>
       <c r="J471" s="1" t="e">
         <f t="shared" si="123"/>
@@ -33352,7 +33353,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="472" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="472" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="G472"/>
       <c r="J472" s="1" t="e">
         <f t="shared" si="123"/>
@@ -33387,7 +33388,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="473" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="473" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="G473"/>
       <c r="J473" s="1" t="e">
         <f t="shared" si="123"/>
@@ -33422,7 +33423,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="474" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="474" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="G474"/>
       <c r="J474" s="1" t="e">
         <f t="shared" si="123"/>
@@ -33457,7 +33458,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="475" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="475" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="G475"/>
       <c r="J475" s="1" t="e">
         <f t="shared" si="123"/>
@@ -33492,7 +33493,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="476" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="476" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="G476"/>
       <c r="J476" s="1" t="e">
         <f t="shared" si="123"/>
@@ -33527,7 +33528,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="477" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="477" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="J477" s="1" t="e">
         <f t="shared" si="123"/>
         <v>#VALUE!</v>
@@ -33561,7 +33562,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="478" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="478" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="J478" s="1" t="e">
         <f t="shared" si="123"/>
         <v>#VALUE!</v>
@@ -33595,7 +33596,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="479" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="479" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="J479" s="1" t="e">
         <f t="shared" si="123"/>
         <v>#VALUE!</v>
@@ -33629,7 +33630,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="480" spans="7:17" x14ac:dyDescent="0.25">
+    <row r="480" spans="7:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="J480" s="1" t="e">
         <f t="shared" si="123"/>
         <v>#VALUE!</v>
@@ -33663,7 +33664,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="481" spans="10:17" x14ac:dyDescent="0.25">
+    <row r="481" spans="10:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="J481" s="1" t="e">
         <f t="shared" si="123"/>
         <v>#VALUE!</v>
@@ -33698,7 +33699,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R481" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:R481" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Panulirus argus"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>